<commit_message>
Planilha de cálculo em PDF; meses em português e índices SELIC marcados para conferência
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsu4pqVYrCnjVCP87tgm6x
</commit_message>
<xml_diff>
--- a/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
+++ b/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="63">
   <si>
     <t xml:space="preserve">PLANILHA DE CÁLCULO – CUMPRIMENTO DE SENTENÇA</t>
   </si>
@@ -239,13 +239,10 @@
     <t xml:space="preserve">Observação</t>
   </si>
   <si>
-    <t xml:space="preserve">Oficial</t>
-  </si>
-  <si>
     <t xml:space="preserve">Conferir</t>
   </si>
   <si>
-    <t xml:space="preserve">Fonte secundária – confirmar no BCB</t>
+    <t xml:space="preserve">Confirmar na série oficial do BCB</t>
   </si>
   <si>
     <t xml:space="preserve">Estimativa</t>
@@ -270,7 +267,7 @@
     <numFmt numFmtId="166" formatCode="&quot;R$ &quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.000000"/>
     <numFmt numFmtId="168" formatCode="0%"/>
-    <numFmt numFmtId="169" formatCode="mmm/yyyy"/>
+    <numFmt numFmtId="169" formatCode="[$-416]mmm/yyyy"/>
     <numFmt numFmtId="170" formatCode="0.00%"/>
     <numFmt numFmtId="171" formatCode="0.0000"/>
     <numFmt numFmtId="172" formatCode="0.0000%"/>
@@ -442,7 +439,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -535,15 +532,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1267,7 +1260,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1334,10 +1327,12 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A5,0),Resumo!$C$12)-MAX(A5-1,Resumo!$C$11))/DAY(EOMONTH(A5,0))</f>
         <v>0</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="10"/>
+      <c r="F5" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
@@ -1354,10 +1349,12 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A6,0),Resumo!$C$12)-MAX(A6-1,Resumo!$C$11))/DAY(EOMONTH(A6,0))</f>
         <v>0</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="10"/>
+      <c r="F6" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
@@ -1374,10 +1371,12 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A7,0),Resumo!$C$12)-MAX(A7-1,Resumo!$C$11))/DAY(EOMONTH(A7,0))</f>
         <v>0</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="10"/>
+      <c r="F7" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
@@ -1394,16 +1393,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A8,0),Resumo!$C$12)-MAX(A8-1,Resumo!$C$11))/DAY(EOMONTH(A8,0))</f>
         <v>0</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="10"/>
+      <c r="F8" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="n">
         <v>46023</v>
       </c>
-      <c r="B9" s="25" t="n">
+      <c r="B9" s="23" t="n">
         <v>0.0116</v>
       </c>
       <c r="C9" s="24" t="n">
@@ -1414,18 +1415,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A9,0),Resumo!$C$12)-MAX(A9-1,Resumo!$C$11))/DAY(EOMONTH(A9,0))</f>
         <v>0</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>46054</v>
       </c>
-      <c r="B10" s="25" t="n">
+      <c r="B10" s="23" t="n">
         <v>0.01</v>
       </c>
       <c r="C10" s="24" t="n">
@@ -1436,18 +1437,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A10,0),Resumo!$C$12)-MAX(A10-1,Resumo!$C$11))/DAY(EOMONTH(A10,0))</f>
         <v>0</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>46082</v>
       </c>
-      <c r="B11" s="25" t="n">
+      <c r="B11" s="23" t="n">
         <v>0.0121</v>
       </c>
       <c r="C11" s="24" t="n">
@@ -1458,18 +1459,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A11,0),Resumo!$C$12)-MAX(A11-1,Resumo!$C$11))/DAY(EOMONTH(A11,0))</f>
         <v>0</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F11" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>46113</v>
       </c>
-      <c r="B12" s="25" t="n">
+      <c r="B12" s="23" t="n">
         <v>0.0109</v>
       </c>
       <c r="C12" s="24" t="n">
@@ -1480,18 +1481,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A12,0),Resumo!$C$12)-MAX(A12-1,Resumo!$C$11))/DAY(EOMONTH(A12,0))</f>
         <v>0</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="n">
         <v>46143</v>
       </c>
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="23" t="n">
         <v>0.0107</v>
       </c>
       <c r="C13" s="24" t="n">
@@ -1502,18 +1503,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A13,0),Resumo!$C$12)-MAX(A13-1,Resumo!$C$11))/DAY(EOMONTH(A13,0))</f>
         <v>0</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="n">
         <v>46174</v>
       </c>
-      <c r="B14" s="25" t="n">
+      <c r="B14" s="23" t="n">
         <v>0.0112</v>
       </c>
       <c r="C14" s="24" t="n">
@@ -1524,18 +1525,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A14,0),Resumo!$C$12)-MAX(A14-1,Resumo!$C$11))/DAY(EOMONTH(A14,0))</f>
         <v>0</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="n">
         <v>46204</v>
       </c>
-      <c r="B15" s="25" t="n">
+      <c r="B15" s="23" t="n">
         <v>0.0122</v>
       </c>
       <c r="C15" s="24" t="n">
@@ -1546,18 +1547,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A15,0),Resumo!$C$12)-MAX(A15-1,Resumo!$C$11))/DAY(EOMONTH(A15,0))</f>
         <v>0.032258064516129</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="22" t="n">
         <v>46235</v>
       </c>
-      <c r="B16" s="25" t="n">
+      <c r="B16" s="23" t="n">
         <v>0.0099</v>
       </c>
       <c r="C16" s="24" t="n">
@@ -1568,18 +1569,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A16,0),Resumo!$C$12)-MAX(A16-1,Resumo!$C$11))/DAY(EOMONTH(A16,0))</f>
         <v>1</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>58</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="n">
         <v>46266</v>
       </c>
-      <c r="B17" s="25" t="n">
+      <c r="B17" s="23" t="n">
         <v>0.0099</v>
       </c>
       <c r="C17" s="24" t="n">
@@ -1590,18 +1591,18 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A17,0),Resumo!$C$12)-MAX(A17-1,Resumo!$C$11))/DAY(EOMONTH(A17,0))</f>
         <v>1</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>60</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="n">
         <v>46296</v>
       </c>
-      <c r="B18" s="25" t="n">
+      <c r="B18" s="23" t="n">
         <v>0.0099</v>
       </c>
       <c r="C18" s="24" t="n">
@@ -1612,37 +1613,37 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$11))/DAY(EOMONTH(A18,0))</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" s="10" t="s">
         <v>60</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B20" s="12"/>
-      <c r="C20" s="27" t="n">
+      <c r="C20" s="26" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*C5:C18)))</f>
         <v>1.14407885292862</v>
       </c>
-      <c r="D20" s="27" t="n">
+      <c r="D20" s="26" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*D5:D18)))</f>
         <v>1.03007451562321</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" s="12"/>
-      <c r="C21" s="28" t="n">
+      <c r="C21" s="27" t="n">
         <f aca="false">C20-1</f>
         <v>0.144078852928615</v>
       </c>
-      <c r="D21" s="28" t="n">
+      <c r="D21" s="27" t="n">
         <f aca="false">D20-1</f>
         <v>0.0300745156232065</v>
       </c>
@@ -1653,11 +1654,11 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
-    <oddFooter/>
+    <oddFooter>&amp;C&amp;8 &amp;K123bb8Rua Rio Grande do Sul, 1641, bairro São Miguel, CEP: 64.130-000, Miguel Alves-PI – (86) 9 7400-9869 – paduanetojus@gmail.com</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza cálculo com a data da citação (17/11/2025)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsu4pqVYrCnjVCP87tgm6x
</commit_message>
<xml_diff>
--- a/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
+++ b/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
@@ -20,49 +20,6 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="C10" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">CONFERIR: data da citação nos autos (juntada do AR/ciência eletrônica). A data aqui lançada é provisória e altera todo o cálculo da restituição.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>1</xdr:col>
-                <xdr:colOff>42</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>4</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>2</xdr:col>
-                <xdr:colOff>-154</xdr:colOff>
-                <xdr:row>5</xdr:row>
-                <xdr:rowOff>11</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="63">
   <si>
@@ -210,7 +167,7 @@
     <t xml:space="preserve">5. Custas processuais: a cargo dos executados, conforme a conta da Secretaria; não integram o crédito da exequente, beneficiária da gratuidade.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Células em amarelo devem ser conferidas antes do protocolo (data da citação e índices SELIC não oficiais).</t>
+    <t xml:space="preserve">6. Células em amarelo devem ser conferidas antes do protocolo (índices SELIC não confirmados na série oficial).</t>
   </si>
   <si>
     <t xml:space="preserve">TABELA DA TAXA SELIC ACUMULADA NO MÊS (BCB – SGS 4390)</t>
@@ -272,7 +229,7 @@
     <numFmt numFmtId="171" formatCode="0.0000"/>
     <numFmt numFmtId="172" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -329,11 +286,6 @@
       <name val="Lora"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -439,7 +391,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -460,10 +412,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -520,11 +468,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -898,7 +846,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>45950</v>
+        <v>45978</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
@@ -908,23 +856,23 @@
       <c r="B11" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="5" t="n">
         <v>46233</v>
       </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="5" t="n">
         <v>46325</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
@@ -991,98 +939,98 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="7" t="n">
         <v>33247.41</v>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="8" t="n">
         <f aca="false">SELIC!$C$20</f>
-        <v>1.14407885292862</v>
-      </c>
-      <c r="E19" s="8" t="n">
+        <v>1.13219993830237</v>
+      </c>
+      <c r="E19" s="7" t="n">
         <f aca="false">ROUND(C19*D19,2)</f>
-        <v>38037.66</v>
-      </c>
-      <c r="F19" s="10" t="s">
+        <v>37642.72</v>
+      </c>
+      <c r="F19" s="9" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="6" t="s">
         <v>24</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="8" t="n">
         <f aca="false">SELIC!$D$20</f>
         <v>1.03007451562321</v>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="7" t="n">
         <f aca="false">ROUND(C20*D20,2)</f>
         <v>2060.15</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="9" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="6" t="s">
         <v>27</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="10" t="n">
         <f aca="false">C19+C20</f>
         <v>35247.41</v>
       </c>
-      <c r="D21" s="12"/>
-      <c r="E21" s="13" t="n">
+      <c r="D21" s="11"/>
+      <c r="E21" s="12" t="n">
         <f aca="false">E19+E20</f>
-        <v>40097.81</v>
-      </c>
-      <c r="F21" s="12"/>
+        <v>39702.87</v>
+      </c>
+      <c r="F21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="6" t="s">
         <v>29</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="14" t="n">
+      <c r="C22" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="D22" s="7"/>
-      <c r="E22" s="8" t="n">
+      <c r="D22" s="6"/>
+      <c r="E22" s="7" t="n">
         <f aca="false">ROUND(E21*C22,2)</f>
-        <v>4009.78</v>
-      </c>
-      <c r="F22" s="10" t="s">
+        <v>3970.29</v>
+      </c>
+      <c r="F22" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15"/>
-      <c r="B23" s="16" t="s">
+      <c r="A23" s="14"/>
+      <c r="B23" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="17" t="n">
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="16" t="n">
         <f aca="false">E21+E22</f>
-        <v>44107.59</v>
-      </c>
-      <c r="F23" s="15"/>
+        <v>43673.16</v>
+      </c>
+      <c r="F23" s="14"/>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
@@ -1101,125 +1049,125 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="6" t="s">
         <v>36</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C26" s="4"/>
-      <c r="D26" s="14" t="n">
+      <c r="D26" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="E26" s="8" t="n">
+      <c r="E26" s="7" t="n">
         <f aca="false">ROUND($E$23*D26,2)</f>
-        <v>4410.76</v>
-      </c>
-      <c r="F26" s="10" t="s">
+        <v>4367.32</v>
+      </c>
+      <c r="F26" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="6" t="s">
         <v>39</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C27" s="4"/>
-      <c r="D27" s="14" t="n">
+      <c r="D27" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="E27" s="8" t="n">
+      <c r="E27" s="7" t="n">
         <f aca="false">ROUND($E$23*D27,2)</f>
-        <v>4410.76</v>
-      </c>
-      <c r="F27" s="10" t="s">
+        <v>4367.32</v>
+      </c>
+      <c r="F27" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15"/>
-      <c r="B28" s="18" t="s">
+      <c r="A28" s="14"/>
+      <c r="B28" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="17" t="n">
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="16" t="n">
         <f aca="false">E23+E26+E27</f>
-        <v>52929.11</v>
-      </c>
-      <c r="F28" s="15"/>
+        <v>52407.8</v>
+      </c>
+      <c r="F28" s="14"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="s">
+      <c r="A30" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="s">
+      <c r="A31" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="s">
+      <c r="A32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
+      <c r="A33" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
+      <c r="A34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -1252,8 +1200,7 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 &amp;K123bb8Rua Rio Grande do Sul, 1641, bairro São Miguel, CEP: 64.130-000, Miguel Alves-PI – (86) 9 7400-9869 – paduanetojus@gmail.com</oddFooter>
   </headerFooter>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1273,24 +1220,24 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -1313,310 +1260,310 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="n">
+      <c r="A5" s="21" t="n">
         <v>45901</v>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="22" t="n">
         <v>0.0122</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A5,0),Resumo!$C$12)-MAX(A5-1,Resumo!$C$10))/DAY(EOMONTH(A5,0))</f>
         <v>0</v>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A5,0),Resumo!$C$12)-MAX(A5-1,Resumo!$C$11))/DAY(EOMONTH(A5,0))</f>
         <v>0</v>
       </c>
-      <c r="E5" s="25" t="s">
+      <c r="E5" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="n">
+      <c r="A6" s="21" t="n">
         <v>45931</v>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="22" t="n">
         <v>0.0128</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A6,0),Resumo!$C$12)-MAX(A6-1,Resumo!$C$10))/DAY(EOMONTH(A6,0))</f>
-        <v>0.354838709677419</v>
-      </c>
-      <c r="D6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A6,0),Resumo!$C$12)-MAX(A6-1,Resumo!$C$11))/DAY(EOMONTH(A6,0))</f>
         <v>0</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="n">
+      <c r="A7" s="21" t="n">
         <v>45962</v>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="22" t="n">
         <v>0.0105</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A7,0),Resumo!$C$12)-MAX(A7-1,Resumo!$C$10))/DAY(EOMONTH(A7,0))</f>
-        <v>1</v>
-      </c>
-      <c r="D7" s="24" t="n">
+        <v>0.433333333333333</v>
+      </c>
+      <c r="D7" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A7,0),Resumo!$C$12)-MAX(A7-1,Resumo!$C$11))/DAY(EOMONTH(A7,0))</f>
         <v>0</v>
       </c>
-      <c r="E7" s="25" t="s">
+      <c r="E7" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="n">
+      <c r="A8" s="21" t="n">
         <v>45992</v>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="22" t="n">
         <v>0.0122</v>
       </c>
-      <c r="C8" s="24" t="n">
+      <c r="C8" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A8,0),Resumo!$C$12)-MAX(A8-1,Resumo!$C$10))/DAY(EOMONTH(A8,0))</f>
         <v>1</v>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A8,0),Resumo!$C$12)-MAX(A8-1,Resumo!$C$11))/DAY(EOMONTH(A8,0))</f>
         <v>0</v>
       </c>
-      <c r="E8" s="25" t="s">
+      <c r="E8" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="22" t="n">
+      <c r="A9" s="21" t="n">
         <v>46023</v>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="22" t="n">
         <v>0.0116</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A9,0),Resumo!$C$12)-MAX(A9-1,Resumo!$C$10))/DAY(EOMONTH(A9,0))</f>
         <v>1</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A9,0),Resumo!$C$12)-MAX(A9-1,Resumo!$C$11))/DAY(EOMONTH(A9,0))</f>
         <v>0</v>
       </c>
-      <c r="E9" s="25" t="s">
+      <c r="E9" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="22" t="n">
+      <c r="A10" s="21" t="n">
         <v>46054</v>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C10" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A10,0),Resumo!$C$12)-MAX(A10-1,Resumo!$C$10))/DAY(EOMONTH(A10,0))</f>
         <v>1</v>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A10,0),Resumo!$C$12)-MAX(A10-1,Resumo!$C$11))/DAY(EOMONTH(A10,0))</f>
         <v>0</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="n">
+      <c r="A11" s="21" t="n">
         <v>46082</v>
       </c>
-      <c r="B11" s="23" t="n">
+      <c r="B11" s="22" t="n">
         <v>0.0121</v>
       </c>
-      <c r="C11" s="24" t="n">
+      <c r="C11" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A11,0),Resumo!$C$12)-MAX(A11-1,Resumo!$C$10))/DAY(EOMONTH(A11,0))</f>
         <v>1</v>
       </c>
-      <c r="D11" s="24" t="n">
+      <c r="D11" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A11,0),Resumo!$C$12)-MAX(A11-1,Resumo!$C$11))/DAY(EOMONTH(A11,0))</f>
         <v>0</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22" t="n">
+      <c r="A12" s="21" t="n">
         <v>46113</v>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="22" t="n">
         <v>0.0109</v>
       </c>
-      <c r="C12" s="24" t="n">
+      <c r="C12" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A12,0),Resumo!$C$12)-MAX(A12-1,Resumo!$C$10))/DAY(EOMONTH(A12,0))</f>
         <v>1</v>
       </c>
-      <c r="D12" s="24" t="n">
+      <c r="D12" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A12,0),Resumo!$C$12)-MAX(A12-1,Resumo!$C$11))/DAY(EOMONTH(A12,0))</f>
         <v>0</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="22" t="n">
+      <c r="A13" s="21" t="n">
         <v>46143</v>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="22" t="n">
         <v>0.0107</v>
       </c>
-      <c r="C13" s="24" t="n">
+      <c r="C13" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A13,0),Resumo!$C$12)-MAX(A13-1,Resumo!$C$10))/DAY(EOMONTH(A13,0))</f>
         <v>1</v>
       </c>
-      <c r="D13" s="24" t="n">
+      <c r="D13" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A13,0),Resumo!$C$12)-MAX(A13-1,Resumo!$C$11))/DAY(EOMONTH(A13,0))</f>
         <v>0</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="n">
+      <c r="A14" s="21" t="n">
         <v>46174</v>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="22" t="n">
         <v>0.0112</v>
       </c>
-      <c r="C14" s="24" t="n">
+      <c r="C14" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A14,0),Resumo!$C$12)-MAX(A14-1,Resumo!$C$10))/DAY(EOMONTH(A14,0))</f>
         <v>1</v>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A14,0),Resumo!$C$12)-MAX(A14-1,Resumo!$C$11))/DAY(EOMONTH(A14,0))</f>
         <v>0</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22" t="n">
+      <c r="A15" s="21" t="n">
         <v>46204</v>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="22" t="n">
         <v>0.0122</v>
       </c>
-      <c r="C15" s="24" t="n">
+      <c r="C15" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A15,0),Resumo!$C$12)-MAX(A15-1,Resumo!$C$10))/DAY(EOMONTH(A15,0))</f>
         <v>1</v>
       </c>
-      <c r="D15" s="24" t="n">
+      <c r="D15" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A15,0),Resumo!$C$12)-MAX(A15-1,Resumo!$C$11))/DAY(EOMONTH(A15,0))</f>
         <v>0.032258064516129</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22" t="n">
+      <c r="A16" s="21" t="n">
         <v>46235</v>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="22" t="n">
         <v>0.0099</v>
       </c>
-      <c r="C16" s="24" t="n">
+      <c r="C16" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A16,0),Resumo!$C$12)-MAX(A16-1,Resumo!$C$10))/DAY(EOMONTH(A16,0))</f>
         <v>1</v>
       </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A16,0),Resumo!$C$12)-MAX(A16-1,Resumo!$C$11))/DAY(EOMONTH(A16,0))</f>
         <v>1</v>
       </c>
-      <c r="E16" s="25" t="s">
+      <c r="E16" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="n">
+      <c r="A17" s="21" t="n">
         <v>46266</v>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="22" t="n">
         <v>0.0099</v>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C17" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A17,0),Resumo!$C$12)-MAX(A17-1,Resumo!$C$10))/DAY(EOMONTH(A17,0))</f>
         <v>1</v>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A17,0),Resumo!$C$12)-MAX(A17-1,Resumo!$C$11))/DAY(EOMONTH(A17,0))</f>
         <v>1</v>
       </c>
-      <c r="E17" s="25" t="s">
+      <c r="E17" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22" t="n">
+      <c r="A18" s="21" t="n">
         <v>46296</v>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="22" t="n">
         <v>0.0099</v>
       </c>
-      <c r="C18" s="24" t="n">
+      <c r="C18" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$10))/DAY(EOMONTH(A18,0))</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="D18" s="24" t="n">
+      <c r="D18" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$11))/DAY(EOMONTH(A18,0))</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="E18" s="25" t="s">
+      <c r="E18" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="9" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1624,12 +1571,12 @@
       <c r="A20" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="26" t="n">
+      <c r="B20" s="11"/>
+      <c r="C20" s="25" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*C5:C18)))</f>
-        <v>1.14407885292862</v>
-      </c>
-      <c r="D20" s="26" t="n">
+        <v>1.13219993830237</v>
+      </c>
+      <c r="D20" s="25" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*D5:D18)))</f>
         <v>1.03007451562321</v>
       </c>
@@ -1638,12 +1585,12 @@
       <c r="A21" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="27" t="n">
+      <c r="B21" s="11"/>
+      <c r="C21" s="26" t="n">
         <f aca="false">C20-1</f>
-        <v>0.144078852928615</v>
-      </c>
-      <c r="D21" s="27" t="n">
+        <v>0.13219993830237</v>
+      </c>
+      <c r="D21" s="26" t="n">
         <f aca="false">D20-1</f>
         <v>0.0300745156232065</v>
       </c>

</xml_diff>

<commit_message>
Atualiza SELIC (AASP/CFC: ago/2026 1,09% e set/2026 1,08%) e recalcula
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsu4pqVYrCnjVCP87tgm6x
</commit_message>
<xml_diff>
--- a/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
+++ b/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
   <si>
     <t xml:space="preserve">PLANILHA DE CÁLCULO – CUMPRIMENTO DE SENTENÇA</t>
   </si>
@@ -167,13 +167,13 @@
     <t xml:space="preserve">5. Custas processuais: a cargo dos executados, conforme a conta da Secretaria; não integram o crédito da exequente, beneficiária da gratuidade.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Células em amarelo devem ser conferidas antes do protocolo (índices SELIC não confirmados na série oficial).</t>
+    <t xml:space="preserve">6. Taxas SELIC conforme tabela da AASP/CFC (série BCB 4390). Out/2026 (amarelo) é estimativa: repete a taxa de set/2026, proporcional até 30/10/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">TABELA DA TAXA SELIC ACUMULADA NO MÊS (BCB – SGS 4390)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fração = parcela do mês efetivamente decorrida dentro do período de incidência (pro rata die nos meses inicial e final). Células amarelas: conferir com a série oficial antes do protocolo.</t>
+    <t xml:space="preserve">Fração = parcela do mês efetivamente decorrida dentro do período de incidência (pro rata die nos meses inicial e final). Fonte: AASP/CFC (série BCB 4390). Célula amarela: estimativa.</t>
   </si>
   <si>
     <t xml:space="preserve">Mês</t>
@@ -196,16 +196,13 @@
     <t xml:space="preserve">Observação</t>
   </si>
   <si>
-    <t xml:space="preserve">Conferir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmar na série oficial do BCB</t>
+    <t xml:space="preserve">AASP/CFC</t>
   </si>
   <si>
     <t xml:space="preserve">Estimativa</t>
   </si>
   <si>
-    <t xml:space="preserve">Mês sem dado disponível – substituir pelo índice oficial</t>
+    <t xml:space="preserve">Out/2026 ainda não divulgado – repetida a taxa de set/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Fator acumulado</t>
@@ -391,7 +388,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -480,11 +477,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="170" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -950,11 +951,11 @@
       </c>
       <c r="D19" s="8" t="n">
         <f aca="false">SELIC!$C$20</f>
-        <v>1.13219993830237</v>
+        <v>1.13530961958417</v>
       </c>
       <c r="E19" s="7" t="n">
         <f aca="false">ROUND(C19*D19,2)</f>
-        <v>37642.72</v>
+        <v>37746.1</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>23</v>
@@ -972,11 +973,11 @@
       </c>
       <c r="D20" s="8" t="n">
         <f aca="false">SELIC!$D$20</f>
-        <v>1.03007451562321</v>
+        <v>1.03290370093909</v>
       </c>
       <c r="E20" s="7" t="n">
         <f aca="false">ROUND(C20*D20,2)</f>
-        <v>2060.15</v>
+        <v>2065.81</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>26</v>
@@ -996,7 +997,7 @@
       <c r="D21" s="11"/>
       <c r="E21" s="12" t="n">
         <f aca="false">E19+E20</f>
-        <v>39702.87</v>
+        <v>39811.91</v>
       </c>
       <c r="F21" s="11"/>
     </row>
@@ -1013,7 +1014,7 @@
       <c r="D22" s="6"/>
       <c r="E22" s="7" t="n">
         <f aca="false">ROUND(E21*C22,2)</f>
-        <v>3970.29</v>
+        <v>3981.19</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>31</v>
@@ -1028,7 +1029,7 @@
       <c r="D23" s="14"/>
       <c r="E23" s="16" t="n">
         <f aca="false">E21+E22</f>
-        <v>43673.16</v>
+        <v>43793.1</v>
       </c>
       <c r="F23" s="14"/>
     </row>
@@ -1061,7 +1062,7 @@
       </c>
       <c r="E26" s="7" t="n">
         <f aca="false">ROUND($E$23*D26,2)</f>
-        <v>4367.32</v>
+        <v>4379.31</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>38</v>
@@ -1080,7 +1081,7 @@
       </c>
       <c r="E27" s="7" t="n">
         <f aca="false">ROUND($E$23*D27,2)</f>
-        <v>4367.32</v>
+        <v>4379.31</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>38</v>
@@ -1095,7 +1096,7 @@
       <c r="D28" s="17"/>
       <c r="E28" s="16" t="n">
         <f aca="false">E23+E26+E27</f>
-        <v>52407.8</v>
+        <v>52551.72</v>
       </c>
       <c r="F28" s="14"/>
     </row>
@@ -1274,12 +1275,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A5,0),Resumo!$C$12)-MAX(A5-1,Resumo!$C$11))/DAY(EOMONTH(A5,0))</f>
         <v>0</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="n">
@@ -1296,12 +1295,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A6,0),Resumo!$C$12)-MAX(A6-1,Resumo!$C$11))/DAY(EOMONTH(A6,0))</f>
         <v>0</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F6" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="n">
@@ -1318,12 +1315,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A7,0),Resumo!$C$12)-MAX(A7-1,Resumo!$C$11))/DAY(EOMONTH(A7,0))</f>
         <v>0</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="n">
@@ -1340,12 +1335,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A8,0),Resumo!$C$12)-MAX(A8-1,Resumo!$C$11))/DAY(EOMONTH(A8,0))</f>
         <v>0</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="n">
@@ -1362,12 +1355,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A9,0),Resumo!$C$12)-MAX(A9-1,Resumo!$C$11))/DAY(EOMONTH(A9,0))</f>
         <v>0</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="n">
@@ -1384,12 +1375,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A10,0),Resumo!$C$12)-MAX(A10-1,Resumo!$C$11))/DAY(EOMONTH(A10,0))</f>
         <v>0</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="n">
@@ -1406,12 +1395,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A11,0),Resumo!$C$12)-MAX(A11-1,Resumo!$C$11))/DAY(EOMONTH(A11,0))</f>
         <v>0</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="n">
@@ -1428,12 +1415,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A12,0),Resumo!$C$12)-MAX(A12-1,Resumo!$C$11))/DAY(EOMONTH(A12,0))</f>
         <v>0</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="n">
@@ -1450,12 +1435,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A13,0),Resumo!$C$12)-MAX(A13-1,Resumo!$C$11))/DAY(EOMONTH(A13,0))</f>
         <v>0</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="n">
@@ -1472,12 +1455,10 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A14,0),Resumo!$C$12)-MAX(A14-1,Resumo!$C$11))/DAY(EOMONTH(A14,0))</f>
         <v>0</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="n">
@@ -1494,19 +1475,17 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A15,0),Resumo!$C$12)-MAX(A15-1,Resumo!$C$11))/DAY(EOMONTH(A15,0))</f>
         <v>0.032258064516129</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>58</v>
-      </c>
+      <c r="F15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="n">
         <v>46235</v>
       </c>
       <c r="B16" s="22" t="n">
-        <v>0.0099</v>
+        <v>0.0109</v>
       </c>
       <c r="C16" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A16,0),Resumo!$C$12)-MAX(A16-1,Resumo!$C$10))/DAY(EOMONTH(A16,0))</f>
@@ -1516,19 +1495,17 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A16,0),Resumo!$C$12)-MAX(A16-1,Resumo!$C$11))/DAY(EOMONTH(A16,0))</f>
         <v>1</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="E16" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F16" s="9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="n">
         <v>46266</v>
       </c>
       <c r="B17" s="22" t="n">
-        <v>0.0099</v>
+        <v>0.0108</v>
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A17,0),Resumo!$C$12)-MAX(A17-1,Resumo!$C$10))/DAY(EOMONTH(A17,0))</f>
@@ -1538,19 +1515,17 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A17,0),Resumo!$C$12)-MAX(A17-1,Resumo!$C$11))/DAY(EOMONTH(A17,0))</f>
         <v>1</v>
       </c>
-      <c r="E17" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>60</v>
-      </c>
+      <c r="E17" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="n">
         <v>46296</v>
       </c>
-      <c r="B18" s="22" t="n">
-        <v>0.0099</v>
+      <c r="B18" s="24" t="n">
+        <v>0.0108</v>
       </c>
       <c r="C18" s="23" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$10))/DAY(EOMONTH(A18,0))</f>
@@ -1560,39 +1535,39 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$11))/DAY(EOMONTH(A18,0))</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="25" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B20" s="11"/>
-      <c r="C20" s="25" t="n">
+      <c r="C20" s="26" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*C5:C18)))</f>
-        <v>1.13219993830237</v>
-      </c>
-      <c r="D20" s="25" t="n">
+        <v>1.13530961958417</v>
+      </c>
+      <c r="D20" s="26" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*D5:D18)))</f>
-        <v>1.03007451562321</v>
+        <v>1.03290370093909</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" s="11"/>
-      <c r="C21" s="26" t="n">
+      <c r="C21" s="27" t="n">
         <f aca="false">C20-1</f>
-        <v>0.13219993830237</v>
-      </c>
-      <c r="D21" s="26" t="n">
+        <v>0.135309619584169</v>
+      </c>
+      <c r="D21" s="27" t="n">
         <f aca="false">D20-1</f>
-        <v>0.0300745156232065</v>
+        <v>0.0329037009390918</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Inclui parcelas pagas após o ajuizamento (out/2025 a fev/2026, R$ 125,00 por contrato)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsu4pqVYrCnjVCP87tgm6x
</commit_message>
<xml_diff>
--- a/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
+++ b/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Resumo" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="SELIC" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Pagamentos posteriores" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="80">
   <si>
     <t xml:space="preserve">PLANILHA DE CÁLCULO – CUMPRIMENTO DE SENTENÇA</t>
   </si>
@@ -98,21 +99,30 @@
     <t xml:space="preserve">2</t>
   </si>
   <si>
+    <t xml:space="preserve">Parcelas pagas após o ajuizamento (out/2025 a fev/2026 – 3 contratos × R$ 125,00) – detalhamento na aba "Pagamentos posteriores"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sentença, item I (restituição integral do efetivamente pago); art. 323 do CPC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
     <t xml:space="preserve">Indenização por danos morais</t>
   </si>
   <si>
     <t xml:space="preserve">Sentença, item II – SELIC desde o arbitramento (30/07/2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal da condenação (1 + 2)</t>
-  </si>
-  <si>
     <t xml:space="preserve">4</t>
   </si>
   <si>
+    <t xml:space="preserve">Subtotal da condenação (1 + 2 + 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Honorários advocatícios sucumbenciais – 10% sobre o valor da condenação</t>
   </si>
   <si>
@@ -131,7 +141,7 @@
     <t xml:space="preserve">Valor</t>
   </si>
   <si>
-    <t xml:space="preserve">5</t>
+    <t xml:space="preserve">6</t>
   </si>
   <si>
     <t xml:space="preserve">Multa</t>
@@ -140,7 +150,7 @@
     <t xml:space="preserve">Art. 523, § 1º, CPC</t>
   </si>
   <si>
-    <t xml:space="preserve">6</t>
+    <t xml:space="preserve">7</t>
   </si>
   <si>
     <t xml:space="preserve">Honorários advocatícios da fase de cumprimento</t>
@@ -167,7 +177,10 @@
     <t xml:space="preserve">5. Custas processuais: a cargo dos executados, conforme a conta da Secretaria; não integram o crédito da exequente, beneficiária da gratuidade.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Taxas SELIC conforme tabela da AASP/CFC (série BCB 4390). Out/2026 (amarelo) é estimativa: repete a taxa de set/2026, proporcional até 30/10/2026.</t>
+    <t xml:space="preserve">6. Item 2: parcelas de R$ 125,00 por contrato pagas de out/2025 a fev/2026 (após o ajuizamento), não abrangidas pelo valor fixado na decisão ED; restituição devida por integrar o "valor efetivamente pago" (sentença, item I) e por força do art. 323 do CPC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Taxas SELIC conforme tabela da AASP/CFC (série BCB 4390). Out/2026 (amarelo) é estimativa: repete a taxa de set/2026, proporcional até 30/10/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">TABELA DA TAXA SELIC ACUMULADA NO MÊS (BCB – SGS 4390)</t>
@@ -196,6 +209,15 @@
     <t xml:space="preserve">Observação</t>
   </si>
   <si>
+    <t xml:space="preserve">Aux.: início</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aux.: fim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aux.: dias</t>
+  </si>
+  <si>
     <t xml:space="preserve">AASP/CFC</t>
   </si>
   <si>
@@ -209,13 +231,46 @@
   </si>
   <si>
     <t xml:space="preserve">Variação (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARCELAS PAGAS APÓS O AJUIZAMENTO (26/09/2025) – OUT/2025 A FEV/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parcelas de R$ 125,00 por contrato, com vencimento no dia 15. Termo inicial da SELIC: a data do pagamento ou a citação (17/11/2025), o que for posterior.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Competência</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data do pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor pago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Termo inicial SELIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">522</t>
+  </si>
+  <si>
+    <t xml:space="preserve">523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">524</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="&quot;R$ &quot;#,##0.00"/>
@@ -224,9 +279,10 @@
     <numFmt numFmtId="169" formatCode="[$-416]mmm/yyyy"/>
     <numFmt numFmtId="170" formatCode="0.00%"/>
     <numFmt numFmtId="171" formatCode="0.0000"/>
-    <numFmt numFmtId="172" formatCode="0.0000%"/>
+    <numFmt numFmtId="172" formatCode="0"/>
+    <numFmt numFmtId="173" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,6 +355,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF888888"/>
+      <name val="Lora"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -388,7 +451,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -485,6 +548,14 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="170" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -497,7 +568,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -795,7 +870,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -969,103 +1044,107 @@
         <v>25</v>
       </c>
       <c r="C20" s="7" t="n">
+        <f aca="false">'Pagamentos posteriores'!D20</f>
+        <v>1875</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <f aca="false">E20/C20</f>
+        <v>1.12048</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <f aca="false">'Pagamentos posteriores'!G20</f>
+        <v>2100.9</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="7" t="n">
         <v>2000</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D21" s="8" t="n">
         <f aca="false">SELIC!$D$20</f>
         <v>1.03290370093909</v>
       </c>
-      <c r="E20" s="7" t="n">
-        <f aca="false">ROUND(C20*D20,2)</f>
+      <c r="E21" s="7" t="n">
+        <f aca="false">ROUND(C21*D21,2)</f>
         <v>2065.81</v>
       </c>
-      <c r="F20" s="9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <f aca="false">C19+C20</f>
-        <v>35247.41</v>
-      </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="12" t="n">
-        <f aca="false">E19+E20</f>
-        <v>39811.91</v>
-      </c>
-      <c r="F21" s="11"/>
-    </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F21" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="13" t="n">
+      <c r="B22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <f aca="false">SUM(C19:C21)</f>
+        <v>37122.41</v>
+      </c>
+      <c r="D22" s="11"/>
+      <c r="E22" s="12" t="n">
+        <f aca="false">SUM(E19:E21)</f>
+        <v>41912.81</v>
+      </c>
+      <c r="F22" s="11"/>
+    </row>
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="7" t="n">
-        <f aca="false">ROUND(E21*C22,2)</f>
-        <v>3981.19</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14"/>
-      <c r="B23" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="16" t="n">
-        <f aca="false">E21+E22</f>
-        <v>43793.1</v>
-      </c>
-      <c r="F23" s="14"/>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2" t="s">
+      <c r="D23" s="6"/>
+      <c r="E23" s="7" t="n">
+        <f aca="false">ROUND(E22*C23,2)</f>
+        <v>4191.28</v>
+      </c>
+      <c r="F23" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E25" s="2" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14"/>
+      <c r="B24" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="16" t="n">
+        <f aca="false">E22+E23</f>
+        <v>46104.09</v>
+      </c>
+      <c r="F24" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="13" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <f aca="false">ROUND($E$23*D26,2)</f>
-        <v>4379.31</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1080,49 +1159,58 @@
         <v>0.1</v>
       </c>
       <c r="E27" s="7" t="n">
-        <f aca="false">ROUND($E$23*D27,2)</f>
-        <v>4379.31</v>
+        <f aca="false">ROUND($E$24*D27,2)</f>
+        <v>4610.41</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14"/>
-      <c r="B28" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="16" t="n">
-        <f aca="false">E23+E26+E27</f>
-        <v>52551.72</v>
-      </c>
-      <c r="F28" s="14"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="18" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-    </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
+      <c r="B28" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E28" s="7" t="n">
+        <f aca="false">ROUND($E$24*D28,2)</f>
+        <v>4610.41</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14"/>
+      <c r="B29" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="16" t="n">
+        <f aca="false">E24+E27+E28</f>
+        <v>55324.91</v>
+      </c>
+      <c r="F29" s="14"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1132,7 +1220,7 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1142,7 +1230,7 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -1152,7 +1240,7 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -1162,7 +1250,7 @@
     </row>
     <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -1170,8 +1258,28 @@
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
     </row>
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+    </row>
+    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+    </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="C9:F9"/>
@@ -1182,17 +1290,18 @@
     <mergeCell ref="C14:F14"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="C16:F16"/>
-    <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:D29"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A38:F38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
@@ -1210,7 +1319,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -1218,11 +1327,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1232,7 +1343,7 @@
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B2" s="20"/>
       <c r="C2" s="20"/>
@@ -1242,22 +1353,31 @@
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1276,9 +1396,21 @@
         <v>0</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F5" s="9"/>
+      <c r="G5" s="24" t="n">
+        <f aca="false">A5-1</f>
+        <v>45900</v>
+      </c>
+      <c r="H5" s="24" t="n">
+        <f aca="false">EOMONTH(A5,0)</f>
+        <v>45930</v>
+      </c>
+      <c r="I5" s="25" t="n">
+        <f aca="false">DAY(H5)</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="n">
@@ -1296,9 +1428,21 @@
         <v>0</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F6" s="9"/>
+      <c r="G6" s="24" t="n">
+        <f aca="false">A6-1</f>
+        <v>45930</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <f aca="false">EOMONTH(A6,0)</f>
+        <v>45961</v>
+      </c>
+      <c r="I6" s="25" t="n">
+        <f aca="false">DAY(H6)</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="n">
@@ -1316,9 +1460,21 @@
         <v>0</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F7" s="9"/>
+      <c r="G7" s="24" t="n">
+        <f aca="false">A7-1</f>
+        <v>45961</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <f aca="false">EOMONTH(A7,0)</f>
+        <v>45991</v>
+      </c>
+      <c r="I7" s="25" t="n">
+        <f aca="false">DAY(H7)</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="n">
@@ -1336,9 +1492,21 @@
         <v>0</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F8" s="9"/>
+      <c r="G8" s="24" t="n">
+        <f aca="false">A8-1</f>
+        <v>45991</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <f aca="false">EOMONTH(A8,0)</f>
+        <v>46022</v>
+      </c>
+      <c r="I8" s="25" t="n">
+        <f aca="false">DAY(H8)</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="n">
@@ -1356,9 +1524,21 @@
         <v>0</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F9" s="9"/>
+      <c r="G9" s="24" t="n">
+        <f aca="false">A9-1</f>
+        <v>46022</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <f aca="false">EOMONTH(A9,0)</f>
+        <v>46053</v>
+      </c>
+      <c r="I9" s="25" t="n">
+        <f aca="false">DAY(H9)</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="n">
@@ -1376,9 +1556,21 @@
         <v>0</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F10" s="9"/>
+      <c r="G10" s="24" t="n">
+        <f aca="false">A10-1</f>
+        <v>46053</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <f aca="false">EOMONTH(A10,0)</f>
+        <v>46081</v>
+      </c>
+      <c r="I10" s="25" t="n">
+        <f aca="false">DAY(H10)</f>
+        <v>28</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="n">
@@ -1396,9 +1588,21 @@
         <v>0</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F11" s="9"/>
+      <c r="G11" s="24" t="n">
+        <f aca="false">A11-1</f>
+        <v>46081</v>
+      </c>
+      <c r="H11" s="24" t="n">
+        <f aca="false">EOMONTH(A11,0)</f>
+        <v>46112</v>
+      </c>
+      <c r="I11" s="25" t="n">
+        <f aca="false">DAY(H11)</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="n">
@@ -1416,9 +1620,21 @@
         <v>0</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F12" s="9"/>
+      <c r="G12" s="24" t="n">
+        <f aca="false">A12-1</f>
+        <v>46112</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <f aca="false">EOMONTH(A12,0)</f>
+        <v>46142</v>
+      </c>
+      <c r="I12" s="25" t="n">
+        <f aca="false">DAY(H12)</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="n">
@@ -1436,9 +1652,21 @@
         <v>0</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F13" s="9"/>
+      <c r="G13" s="24" t="n">
+        <f aca="false">A13-1</f>
+        <v>46142</v>
+      </c>
+      <c r="H13" s="24" t="n">
+        <f aca="false">EOMONTH(A13,0)</f>
+        <v>46173</v>
+      </c>
+      <c r="I13" s="25" t="n">
+        <f aca="false">DAY(H13)</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="n">
@@ -1456,9 +1684,21 @@
         <v>0</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F14" s="9"/>
+      <c r="G14" s="24" t="n">
+        <f aca="false">A14-1</f>
+        <v>46173</v>
+      </c>
+      <c r="H14" s="24" t="n">
+        <f aca="false">EOMONTH(A14,0)</f>
+        <v>46203</v>
+      </c>
+      <c r="I14" s="25" t="n">
+        <f aca="false">DAY(H14)</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="n">
@@ -1476,9 +1716,21 @@
         <v>0.032258064516129</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F15" s="9"/>
+      <c r="G15" s="24" t="n">
+        <f aca="false">A15-1</f>
+        <v>46203</v>
+      </c>
+      <c r="H15" s="24" t="n">
+        <f aca="false">EOMONTH(A15,0)</f>
+        <v>46234</v>
+      </c>
+      <c r="I15" s="25" t="n">
+        <f aca="false">DAY(H15)</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="n">
@@ -1496,9 +1748,21 @@
         <v>1</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F16" s="9"/>
+      <c r="G16" s="24" t="n">
+        <f aca="false">A16-1</f>
+        <v>46234</v>
+      </c>
+      <c r="H16" s="24" t="n">
+        <f aca="false">EOMONTH(A16,0)</f>
+        <v>46265</v>
+      </c>
+      <c r="I16" s="25" t="n">
+        <f aca="false">DAY(H16)</f>
+        <v>31</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="n">
@@ -1516,15 +1780,27 @@
         <v>1</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F17" s="9"/>
+      <c r="G17" s="24" t="n">
+        <f aca="false">A17-1</f>
+        <v>46265</v>
+      </c>
+      <c r="H17" s="24" t="n">
+        <f aca="false">EOMONTH(A17,0)</f>
+        <v>46295</v>
+      </c>
+      <c r="I17" s="25" t="n">
+        <f aca="false">DAY(H17)</f>
+        <v>30</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="n">
         <v>46296</v>
       </c>
-      <c r="B18" s="24" t="n">
+      <c r="B18" s="26" t="n">
         <v>0.0108</v>
       </c>
       <c r="C18" s="23" t="n">
@@ -1535,37 +1811,49 @@
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$11))/DAY(EOMONTH(A18,0))</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="E18" s="25" t="s">
-        <v>58</v>
+      <c r="E18" s="27" t="s">
+        <v>65</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>59</v>
+        <v>66</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <f aca="false">A18-1</f>
+        <v>46295</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <f aca="false">EOMONTH(A18,0)</f>
+        <v>46326</v>
+      </c>
+      <c r="I18" s="25" t="n">
+        <f aca="false">DAY(H18)</f>
+        <v>31</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B20" s="11"/>
-      <c r="C20" s="26" t="n">
+      <c r="C20" s="28" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*C5:C18)))</f>
         <v>1.13530961958417</v>
       </c>
-      <c r="D20" s="26" t="n">
+      <c r="D20" s="28" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*D5:D18)))</f>
         <v>1.03290370093909</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B21" s="11"/>
-      <c r="C21" s="27" t="n">
+      <c r="C21" s="29" t="n">
         <f aca="false">C20-1</f>
         <v>0.135309619584169</v>
       </c>
-      <c r="D21" s="27" t="n">
+      <c r="D21" s="29" t="n">
         <f aca="false">D20-1</f>
         <v>0.0329037009390918</v>
       </c>
@@ -1583,4 +1871,555 @@
     <oddFooter>&amp;C&amp;8 &amp;K123bb8Rua Rio Grande do Sul, 1641, bairro São Miguel, CEP: 64.130-000, Miguel Alves-PI – (86) 9 7400-9869 – paduanetojus@gmail.com</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+    </row>
+    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="21" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="30" t="n">
+        <v>45945</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E5" s="30" t="n">
+        <f aca="false">MAX(C5,Resumo!$C$10)</f>
+        <v>45978</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E5+ABS(SELIC!$G$5:$G$18-E5))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E5+ABS(SELIC!$G$5:$G$18-E5))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.13530961958417</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <f aca="false">ROUND(D5*F5,2)</f>
+        <v>141.91</v>
+      </c>
+      <c r="H5" s="9" t="str">
+        <f aca="false">IF(C5&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>Pago antes da citação – SELIC desde a citação</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="30" t="n">
+        <v>45945</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E6" s="30" t="n">
+        <f aca="false">MAX(C6,Resumo!$C$10)</f>
+        <v>45978</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E6+ABS(SELIC!$G$5:$G$18-E6))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E6+ABS(SELIC!$G$5:$G$18-E6))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.13530961958417</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <f aca="false">ROUND(D6*F6,2)</f>
+        <v>141.91</v>
+      </c>
+      <c r="H6" s="9" t="str">
+        <f aca="false">IF(C6&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>Pago antes da citação – SELIC desde a citação</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="21" t="n">
+        <v>45931</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="30" t="n">
+        <v>45945</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E7" s="30" t="n">
+        <f aca="false">MAX(C7,Resumo!$C$10)</f>
+        <v>45978</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E7+ABS(SELIC!$G$5:$G$18-E7))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E7+ABS(SELIC!$G$5:$G$18-E7))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.13530961958417</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <f aca="false">ROUND(D7*F7,2)</f>
+        <v>141.91</v>
+      </c>
+      <c r="H7" s="9" t="str">
+        <f aca="false">IF(C7&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>Pago antes da citação – SELIC desde a citação</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" s="30" t="n">
+        <v>45976</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E8" s="30" t="n">
+        <f aca="false">MAX(C8,Resumo!$C$10)</f>
+        <v>45978</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E8+ABS(SELIC!$G$5:$G$18-E8))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E8+ABS(SELIC!$G$5:$G$18-E8))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.13530961958417</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <f aca="false">ROUND(D8*F8,2)</f>
+        <v>141.91</v>
+      </c>
+      <c r="H8" s="9" t="str">
+        <f aca="false">IF(C8&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>Pago antes da citação – SELIC desde a citação</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="30" t="n">
+        <v>45976</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E9" s="30" t="n">
+        <f aca="false">MAX(C9,Resumo!$C$10)</f>
+        <v>45978</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E9+ABS(SELIC!$G$5:$G$18-E9))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E9+ABS(SELIC!$G$5:$G$18-E9))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.13530961958417</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <f aca="false">ROUND(D9*F9,2)</f>
+        <v>141.91</v>
+      </c>
+      <c r="H9" s="9" t="str">
+        <f aca="false">IF(C9&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>Pago antes da citação – SELIC desde a citação</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="n">
+        <v>45962</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="30" t="n">
+        <v>45976</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E10" s="30" t="n">
+        <f aca="false">MAX(C10,Resumo!$C$10)</f>
+        <v>45978</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E10+ABS(SELIC!$G$5:$G$18-E10))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E10+ABS(SELIC!$G$5:$G$18-E10))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.13530961958417</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <f aca="false">ROUND(D10*F10,2)</f>
+        <v>141.91</v>
+      </c>
+      <c r="H10" s="9" t="str">
+        <f aca="false">IF(C10&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>Pago antes da citação – SELIC desde a citação</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="30" t="n">
+        <v>46006</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E11" s="30" t="n">
+        <f aca="false">MAX(C11,Resumo!$C$10)</f>
+        <v>46006</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E11+ABS(SELIC!$G$5:$G$18-E11))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E11+ABS(SELIC!$G$5:$G$18-E11))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.12357613787759</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <f aca="false">ROUND(D11*F11,2)</f>
+        <v>140.45</v>
+      </c>
+      <c r="H11" s="9" t="str">
+        <f aca="false">IF(C11&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="30" t="n">
+        <v>46006</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <f aca="false">MAX(C12,Resumo!$C$10)</f>
+        <v>46006</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E12+ABS(SELIC!$G$5:$G$18-E12))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E12+ABS(SELIC!$G$5:$G$18-E12))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.12357613787759</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <f aca="false">ROUND(D12*F12,2)</f>
+        <v>140.45</v>
+      </c>
+      <c r="H12" s="9" t="str">
+        <f aca="false">IF(C12&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13" s="30" t="n">
+        <v>46006</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <f aca="false">MAX(C13,Resumo!$C$10)</f>
+        <v>46006</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E13+ABS(SELIC!$G$5:$G$18-E13))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E13+ABS(SELIC!$G$5:$G$18-E13))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.12357613787759</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <f aca="false">ROUND(D13*F13,2)</f>
+        <v>140.45</v>
+      </c>
+      <c r="H13" s="9" t="str">
+        <f aca="false">IF(C13&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="30" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E14" s="30" t="n">
+        <f aca="false">MAX(C14,Resumo!$C$10)</f>
+        <v>46037</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E14+ABS(SELIC!$G$5:$G$18-E14))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E14+ABS(SELIC!$G$5:$G$18-E14))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.11035030540494</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <f aca="false">ROUND(D14*F14,2)</f>
+        <v>138.79</v>
+      </c>
+      <c r="H14" s="9" t="str">
+        <f aca="false">IF(C14&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="30" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <f aca="false">MAX(C15,Resumo!$C$10)</f>
+        <v>46037</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E15+ABS(SELIC!$G$5:$G$18-E15))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E15+ABS(SELIC!$G$5:$G$18-E15))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.11035030540494</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <f aca="false">ROUND(D15*F15,2)</f>
+        <v>138.79</v>
+      </c>
+      <c r="H15" s="9" t="str">
+        <f aca="false">IF(C15&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="30" t="n">
+        <v>46037</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E16" s="30" t="n">
+        <f aca="false">MAX(C16,Resumo!$C$10)</f>
+        <v>46037</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E16+ABS(SELIC!$G$5:$G$18-E16))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E16+ABS(SELIC!$G$5:$G$18-E16))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.11035030540494</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <f aca="false">ROUND(D16*F16,2)</f>
+        <v>138.79</v>
+      </c>
+      <c r="H16" s="9" t="str">
+        <f aca="false">IF(C16&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="30" t="n">
+        <v>46068</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E17" s="30" t="n">
+        <f aca="false">MAX(C17,Resumo!$C$10)</f>
+        <v>46068</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E17+ABS(SELIC!$G$5:$G$18-E17))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E17+ABS(SELIC!$G$5:$G$18-E17))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.09788773419655</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <f aca="false">ROUND(D17*F17,2)</f>
+        <v>137.24</v>
+      </c>
+      <c r="H17" s="9" t="str">
+        <f aca="false">IF(C17&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>46068</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E18" s="30" t="n">
+        <f aca="false">MAX(C18,Resumo!$C$10)</f>
+        <v>46068</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E18+ABS(SELIC!$G$5:$G$18-E18))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E18+ABS(SELIC!$G$5:$G$18-E18))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.09788773419655</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <f aca="false">ROUND(D18*F18,2)</f>
+        <v>137.24</v>
+      </c>
+      <c r="H18" s="9" t="str">
+        <f aca="false">IF(C18&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" s="30" t="n">
+        <v>46068</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>125</v>
+      </c>
+      <c r="E19" s="30" t="n">
+        <f aca="false">MAX(C19,Resumo!$C$10)</f>
+        <v>46068</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E19+ABS(SELIC!$G$5:$G$18-E19))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E19+ABS(SELIC!$G$5:$G$18-E19))/2))))/2)/SELIC!$I$5:$I$18)))</f>
+        <v>1.09788773419655</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <f aca="false">ROUND(D19*F19,2)</f>
+        <v>137.24</v>
+      </c>
+      <c r="H19" s="9" t="str">
+        <f aca="false">IF(C19&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
+        <v>SELIC desde o pagamento</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="16" t="n">
+        <f aca="false">SUM(D5:D19)</f>
+        <v>1875</v>
+      </c>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="16" t="n">
+        <f aca="false">SUM(G5:G19)</f>
+        <v>2100.9</v>
+      </c>
+      <c r="H20" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Parcelas posteriores ao ajuizamento limitadas a out/2025-jan/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsu4pqVYrCnjVCP87tgm6x
</commit_message>
<xml_diff>
--- a/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
+++ b/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="80">
   <si>
     <t xml:space="preserve">PLANILHA DE CÁLCULO – CUMPRIMENTO DE SENTENÇA</t>
   </si>
@@ -99,7 +99,7 @@
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">Parcelas pagas após o ajuizamento (out/2025 a fev/2026 – 3 contratos × R$ 125,00) – detalhamento na aba "Pagamentos posteriores"</t>
+    <t xml:space="preserve">Parcelas pagas após o ajuizamento (out/2025 a jan/2026 – 3 contratos × R$ 125,00) – detalhamento na aba "Pagamentos posteriores"</t>
   </si>
   <si>
     <t xml:space="preserve">Sentença, item I (restituição integral do efetivamente pago); art. 323 do CPC</t>
@@ -177,7 +177,7 @@
     <t xml:space="preserve">5. Custas processuais: a cargo dos executados, conforme a conta da Secretaria; não integram o crédito da exequente, beneficiária da gratuidade.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Item 2: parcelas de R$ 125,00 por contrato pagas de out/2025 a fev/2026 (após o ajuizamento), não abrangidas pelo valor fixado na decisão ED; restituição devida por integrar o "valor efetivamente pago" (sentença, item I) e por força do art. 323 do CPC.</t>
+    <t xml:space="preserve">6. Item 2: parcelas de R$ 125,00 por contrato pagas de out/2025 a jan/2026 (após o ajuizamento), não abrangidas pelo valor fixado na decisão ED; restituição devida por integrar o "valor efetivamente pago" (sentença, item I) e por força do art. 323 do CPC.</t>
   </si>
   <si>
     <t xml:space="preserve">7. Taxas SELIC conforme tabela da AASP/CFC (série BCB 4390). Out/2026 (amarelo) é estimativa: repete a taxa de set/2026, proporcional até 30/10/2026.</t>
@@ -233,7 +233,7 @@
     <t xml:space="preserve">Variação (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">PARCELAS PAGAS APÓS O AJUIZAMENTO (26/09/2025) – OUT/2025 A FEV/2026</t>
+    <t xml:space="preserve">PARCELAS PAGAS APÓS O AJUIZAMENTO (26/09/2025) – OUT/2025 A JAN/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Parcelas de R$ 125,00 por contrato, com vencimento no dia 15. Termo inicial da SELIC: a data do pagamento ou a citação (17/11/2025), o que for posterior.</t>
@@ -1044,16 +1044,16 @@
         <v>25</v>
       </c>
       <c r="C20" s="7" t="n">
-        <f aca="false">'Pagamentos posteriores'!D20</f>
-        <v>1875</v>
+        <f aca="false">'Pagamentos posteriores'!D17</f>
+        <v>1500</v>
       </c>
       <c r="D20" s="8" t="n">
         <f aca="false">E20/C20</f>
-        <v>1.12048</v>
+        <v>1.12612</v>
       </c>
       <c r="E20" s="7" t="n">
-        <f aca="false">'Pagamentos posteriores'!G20</f>
-        <v>2100.9</v>
+        <f aca="false">'Pagamentos posteriores'!G17</f>
+        <v>1689.18</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>26</v>
@@ -1090,12 +1090,12 @@
       </c>
       <c r="C22" s="10" t="n">
         <f aca="false">SUM(C19:C21)</f>
-        <v>37122.41</v>
+        <v>36747.41</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="12" t="n">
         <f aca="false">SUM(E19:E21)</f>
-        <v>41912.81</v>
+        <v>41501.09</v>
       </c>
       <c r="F22" s="11"/>
     </row>
@@ -1112,7 +1112,7 @@
       <c r="D23" s="6"/>
       <c r="E23" s="7" t="n">
         <f aca="false">ROUND(E22*C23,2)</f>
-        <v>4191.28</v>
+        <v>4150.11</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>34</v>
@@ -1127,7 +1127,7 @@
       <c r="D24" s="14"/>
       <c r="E24" s="16" t="n">
         <f aca="false">E22+E23</f>
-        <v>46104.09</v>
+        <v>45651.2</v>
       </c>
       <c r="F24" s="14"/>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="E27" s="7" t="n">
         <f aca="false">ROUND($E$24*D27,2)</f>
-        <v>4610.41</v>
+        <v>4565.12</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>41</v>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="E28" s="7" t="n">
         <f aca="false">ROUND($E$24*D28,2)</f>
-        <v>4610.41</v>
+        <v>4565.12</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>41</v>
@@ -1194,7 +1194,7 @@
       <c r="D29" s="17"/>
       <c r="E29" s="16" t="n">
         <f aca="false">E24+E27+E28</f>
-        <v>55324.91</v>
+        <v>54781.44</v>
       </c>
       <c r="F29" s="14"/>
     </row>
@@ -1878,7 +1878,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -2302,112 +2302,22 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
-        <v>46054</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C17" s="30" t="n">
-        <v>46068</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>125</v>
-      </c>
-      <c r="E17" s="30" t="n">
-        <f aca="false">MAX(C17,Resumo!$C$10)</f>
-        <v>46068</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E17+ABS(SELIC!$G$5:$G$18-E17))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E17+ABS(SELIC!$G$5:$G$18-E17))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.09788773419655</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <f aca="false">ROUND(D17*F17,2)</f>
-        <v>137.24</v>
-      </c>
-      <c r="H17" s="9" t="str">
-        <f aca="false">IF(C17&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>SELIC desde o pagamento</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
-        <v>46054</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C18" s="30" t="n">
-        <v>46068</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>125</v>
-      </c>
-      <c r="E18" s="30" t="n">
-        <f aca="false">MAX(C18,Resumo!$C$10)</f>
-        <v>46068</v>
-      </c>
-      <c r="F18" s="8" t="n">
-        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E18+ABS(SELIC!$G$5:$G$18-E18))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E18+ABS(SELIC!$G$5:$G$18-E18))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.09788773419655</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <f aca="false">ROUND(D18*F18,2)</f>
-        <v>137.24</v>
-      </c>
-      <c r="H18" s="9" t="str">
-        <f aca="false">IF(C18&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>SELIC desde o pagamento</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
-        <v>46054</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C19" s="30" t="n">
-        <v>46068</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>125</v>
-      </c>
-      <c r="E19" s="30" t="n">
-        <f aca="false">MAX(C19,Resumo!$C$10)</f>
-        <v>46068</v>
-      </c>
-      <c r="F19" s="8" t="n">
-        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E19+ABS(SELIC!$G$5:$G$18-E19))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E19+ABS(SELIC!$G$5:$G$18-E19))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.09788773419655</v>
-      </c>
-      <c r="G19" s="7" t="n">
-        <f aca="false">ROUND(D19*F19,2)</f>
-        <v>137.24</v>
-      </c>
-      <c r="H19" s="9" t="str">
-        <f aca="false">IF(C19&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>SELIC desde o pagamento</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A17" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="16" t="n">
-        <f aca="false">SUM(D5:D19)</f>
-        <v>1875</v>
-      </c>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="16" t="n">
-        <f aca="false">SUM(G5:G19)</f>
-        <v>2100.9</v>
-      </c>
-      <c r="H20" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="16" t="n">
+        <f aca="false">SUM(D5:D16)</f>
+        <v>1500</v>
+      </c>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="16" t="n">
+        <f aca="false">SUM(G5:G16)</f>
+        <v>1689.18</v>
+      </c>
+      <c r="H17" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Recalcula parcelas posteriores (nov/2025-jan/2026) e inclui conferência do relatório de pagamentos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsu4pqVYrCnjVCP87tgm6x
</commit_message>
<xml_diff>
--- a/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
+++ b/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Resumo" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="SELIC" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Pagamentos posteriores" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Conferência" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="99">
   <si>
     <t xml:space="preserve">PLANILHA DE CÁLCULO – CUMPRIMENTO DE SENTENÇA</t>
   </si>
@@ -99,7 +100,7 @@
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">Parcelas pagas após o ajuizamento (out/2025 a jan/2026 – 3 contratos × R$ 125,00) – detalhamento na aba "Pagamentos posteriores"</t>
+    <t xml:space="preserve">Parcelas pagas após o ajuizamento (nov/2025 a jan/2026 – 3 contratos × R$ 125,00) – detalhamento na aba "Pagamentos posteriores"</t>
   </si>
   <si>
     <t xml:space="preserve">Sentença, item I (restituição integral do efetivamente pago); art. 323 do CPC</t>
@@ -177,7 +178,7 @@
     <t xml:space="preserve">5. Custas processuais: a cargo dos executados, conforme a conta da Secretaria; não integram o crédito da exequente, beneficiária da gratuidade.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Item 2: parcelas de R$ 125,00 por contrato pagas de out/2025 a jan/2026 (após o ajuizamento), não abrangidas pelo valor fixado na decisão ED; restituição devida por integrar o "valor efetivamente pago" (sentença, item I) e por força do art. 323 do CPC.</t>
+    <t xml:space="preserve">6. Item 2: parcelas de R$ 125,00 por contrato pagas de nov/2025 a jan/2026, não abrangidas pelo valor fixado na decisão ED, que já inclui os pagamentos até out/2025 (aba "Conferência"); restituição devida por integrar o "valor efetivamente pago" (sentença, item I) e por força do art. 323 do CPC.</t>
   </si>
   <si>
     <t xml:space="preserve">7. Taxas SELIC conforme tabela da AASP/CFC (série BCB 4390). Out/2026 (amarelo) é estimativa: repete a taxa de set/2026, proporcional até 30/10/2026.</t>
@@ -233,10 +234,10 @@
     <t xml:space="preserve">Variação (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">PARCELAS PAGAS APÓS O AJUIZAMENTO (26/09/2025) – OUT/2025 A JAN/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parcelas de R$ 125,00 por contrato, com vencimento no dia 15. Termo inicial da SELIC: a data do pagamento ou a citação (17/11/2025), o que for posterior.</t>
+    <t xml:space="preserve">PARCELAS PAGAS APÓS O AJUIZAMENTO (26/09/2025) – NOV/2025 A JAN/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parcelas de R$ 125,00 por contrato, com vencimento no dia 15. Set/2025 e out/2025 já integram o valor fixado na decisão ED (aba "Conferência"). Termo inicial da SELIC: a data do pagamento ou a citação (17/11/2025), o que for posterior.</t>
   </si>
   <si>
     <t xml:space="preserve">Competência</t>
@@ -264,6 +265,63 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFERÊNCIA DO VALOR FIXADO NA DECISÃO ED (R$ 33.247,41)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relatório "Contas por tipo" da vendedora, emitido em 01/09/2025 (recebimentos até 01/09/2025), conferido linha a linha.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rubrica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrato 522</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrato 523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contrato 524</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sinal (500,00 + 2 × 260,00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parcela negociada PN001 (fev/2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parcelas mensais 001–092 (exceto 062 e 085)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juros por atraso pagos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total por contrato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reconciliação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total do relatório até 01/09/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(+) Parcelas de set/2025 (3 × R$ 125,00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(+) Parcelas de out/2025 (3 × R$ 125,00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(=) Total pago até out/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor fixado na decisão ED (item "e")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diferença</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conclusão: o valor fixado na decisão ED corresponde aos pagamentos até out/2025 (diferença residual de R$ 4,02, compatível com encargos). Por isso, o item 2 do Resumo considera apenas as parcelas de nov/2025 a jan/2026, sem duplicidade. Observação: a parcela 085 (jan/2025) não consta do relatório em nenhum dos três contratos.</t>
   </si>
 </sst>
 </file>
@@ -389,7 +447,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -425,6 +483,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF888888"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF888888"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -451,7 +520,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -574,6 +643,10 @@
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1044,16 +1117,16 @@
         <v>25</v>
       </c>
       <c r="C20" s="7" t="n">
-        <f aca="false">'Pagamentos posteriores'!D17</f>
-        <v>1500</v>
+        <f aca="false">'Pagamentos posteriores'!D14</f>
+        <v>1125</v>
       </c>
       <c r="D20" s="8" t="n">
         <f aca="false">E20/C20</f>
-        <v>1.12612</v>
+        <v>1.12306666666667</v>
       </c>
       <c r="E20" s="7" t="n">
-        <f aca="false">'Pagamentos posteriores'!G17</f>
-        <v>1689.18</v>
+        <f aca="false">'Pagamentos posteriores'!G14</f>
+        <v>1263.45</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>26</v>
@@ -1090,12 +1163,12 @@
       </c>
       <c r="C22" s="10" t="n">
         <f aca="false">SUM(C19:C21)</f>
-        <v>36747.41</v>
+        <v>36372.41</v>
       </c>
       <c r="D22" s="11"/>
       <c r="E22" s="12" t="n">
         <f aca="false">SUM(E19:E21)</f>
-        <v>41501.09</v>
+        <v>41075.36</v>
       </c>
       <c r="F22" s="11"/>
     </row>
@@ -1112,7 +1185,7 @@
       <c r="D23" s="6"/>
       <c r="E23" s="7" t="n">
         <f aca="false">ROUND(E22*C23,2)</f>
-        <v>4150.11</v>
+        <v>4107.54</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>34</v>
@@ -1127,7 +1200,7 @@
       <c r="D24" s="14"/>
       <c r="E24" s="16" t="n">
         <f aca="false">E22+E23</f>
-        <v>45651.2</v>
+        <v>45182.9</v>
       </c>
       <c r="F24" s="14"/>
     </row>
@@ -1160,7 +1233,7 @@
       </c>
       <c r="E27" s="7" t="n">
         <f aca="false">ROUND($E$24*D27,2)</f>
-        <v>4565.12</v>
+        <v>4518.29</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>41</v>
@@ -1179,7 +1252,7 @@
       </c>
       <c r="E28" s="7" t="n">
         <f aca="false">ROUND($E$24*D28,2)</f>
-        <v>4565.12</v>
+        <v>4518.29</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>41</v>
@@ -1194,7 +1267,7 @@
       <c r="D29" s="17"/>
       <c r="E29" s="16" t="n">
         <f aca="false">E24+E27+E28</f>
-        <v>54781.44</v>
+        <v>54219.48</v>
       </c>
       <c r="F29" s="14"/>
     </row>
@@ -1878,7 +1951,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -1943,13 +2016,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>76</v>
       </c>
       <c r="C5" s="30" t="n">
-        <v>45945</v>
+        <v>45976</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>125</v>
@@ -1973,13 +2046,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C6" s="30" t="n">
-        <v>45945</v>
+        <v>45976</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>125</v>
@@ -2003,13 +2076,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="n">
-        <v>45931</v>
+        <v>45962</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C7" s="30" t="n">
-        <v>45945</v>
+        <v>45976</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>125</v>
@@ -2033,118 +2106,118 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>76</v>
       </c>
       <c r="C8" s="30" t="n">
-        <v>45976</v>
+        <v>46006</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>125</v>
       </c>
       <c r="E8" s="30" t="n">
         <f aca="false">MAX(C8,Resumo!$C$10)</f>
-        <v>45978</v>
+        <v>46006</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E8+ABS(SELIC!$G$5:$G$18-E8))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E8+ABS(SELIC!$G$5:$G$18-E8))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.13530961958417</v>
+        <v>1.12357613787759</v>
       </c>
       <c r="G8" s="7" t="n">
         <f aca="false">ROUND(D8*F8,2)</f>
-        <v>141.91</v>
+        <v>140.45</v>
       </c>
       <c r="H8" s="9" t="str">
         <f aca="false">IF(C8&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>Pago antes da citação – SELIC desde a citação</v>
+        <v>SELIC desde o pagamento</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C9" s="30" t="n">
-        <v>45976</v>
+        <v>46006</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>125</v>
       </c>
       <c r="E9" s="30" t="n">
         <f aca="false">MAX(C9,Resumo!$C$10)</f>
-        <v>45978</v>
+        <v>46006</v>
       </c>
       <c r="F9" s="8" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E9+ABS(SELIC!$G$5:$G$18-E9))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E9+ABS(SELIC!$G$5:$G$18-E9))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.13530961958417</v>
+        <v>1.12357613787759</v>
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">ROUND(D9*F9,2)</f>
-        <v>141.91</v>
+        <v>140.45</v>
       </c>
       <c r="H9" s="9" t="str">
         <f aca="false">IF(C9&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>Pago antes da citação – SELIC desde a citação</v>
+        <v>SELIC desde o pagamento</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="n">
-        <v>45962</v>
+        <v>45992</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C10" s="30" t="n">
-        <v>45976</v>
+        <v>46006</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>125</v>
       </c>
       <c r="E10" s="30" t="n">
         <f aca="false">MAX(C10,Resumo!$C$10)</f>
-        <v>45978</v>
+        <v>46006</v>
       </c>
       <c r="F10" s="8" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E10+ABS(SELIC!$G$5:$G$18-E10))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E10+ABS(SELIC!$G$5:$G$18-E10))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.13530961958417</v>
+        <v>1.12357613787759</v>
       </c>
       <c r="G10" s="7" t="n">
         <f aca="false">ROUND(D10*F10,2)</f>
-        <v>141.91</v>
+        <v>140.45</v>
       </c>
       <c r="H10" s="9" t="str">
         <f aca="false">IF(C10&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>Pago antes da citação – SELIC desde a citação</v>
+        <v>SELIC desde o pagamento</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>76</v>
       </c>
       <c r="C11" s="30" t="n">
-        <v>46006</v>
+        <v>46037</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>125</v>
       </c>
       <c r="E11" s="30" t="n">
         <f aca="false">MAX(C11,Resumo!$C$10)</f>
-        <v>46006</v>
+        <v>46037</v>
       </c>
       <c r="F11" s="8" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E11+ABS(SELIC!$G$5:$G$18-E11))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E11+ABS(SELIC!$G$5:$G$18-E11))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.12357613787759</v>
+        <v>1.11035030540494</v>
       </c>
       <c r="G11" s="7" t="n">
         <f aca="false">ROUND(D11*F11,2)</f>
-        <v>140.45</v>
+        <v>138.79</v>
       </c>
       <c r="H11" s="9" t="str">
         <f aca="false">IF(C11&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
@@ -2153,28 +2226,28 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>77</v>
       </c>
       <c r="C12" s="30" t="n">
-        <v>46006</v>
+        <v>46037</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>125</v>
       </c>
       <c r="E12" s="30" t="n">
         <f aca="false">MAX(C12,Resumo!$C$10)</f>
-        <v>46006</v>
+        <v>46037</v>
       </c>
       <c r="F12" s="8" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E12+ABS(SELIC!$G$5:$G$18-E12))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E12+ABS(SELIC!$G$5:$G$18-E12))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.12357613787759</v>
+        <v>1.11035030540494</v>
       </c>
       <c r="G12" s="7" t="n">
         <f aca="false">ROUND(D12*F12,2)</f>
-        <v>140.45</v>
+        <v>138.79</v>
       </c>
       <c r="H12" s="9" t="str">
         <f aca="false">IF(C12&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
@@ -2183,28 +2256,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="n">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>78</v>
       </c>
       <c r="C13" s="30" t="n">
-        <v>46006</v>
+        <v>46037</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>125</v>
       </c>
       <c r="E13" s="30" t="n">
         <f aca="false">MAX(C13,Resumo!$C$10)</f>
-        <v>46006</v>
+        <v>46037</v>
       </c>
       <c r="F13" s="8" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E13+ABS(SELIC!$G$5:$G$18-E13))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E13+ABS(SELIC!$G$5:$G$18-E13))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.12357613787759</v>
+        <v>1.11035030540494</v>
       </c>
       <c r="G13" s="7" t="n">
         <f aca="false">ROUND(D13*F13,2)</f>
-        <v>140.45</v>
+        <v>138.79</v>
       </c>
       <c r="H13" s="9" t="str">
         <f aca="false">IF(C13&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
@@ -2212,112 +2285,22 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C14" s="30" t="n">
-        <v>46037</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>125</v>
-      </c>
-      <c r="E14" s="30" t="n">
-        <f aca="false">MAX(C14,Resumo!$C$10)</f>
-        <v>46037</v>
-      </c>
-      <c r="F14" s="8" t="n">
-        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E14+ABS(SELIC!$G$5:$G$18-E14))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E14+ABS(SELIC!$G$5:$G$18-E14))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.11035030540494</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <f aca="false">ROUND(D14*F14,2)</f>
-        <v>138.79</v>
-      </c>
-      <c r="H14" s="9" t="str">
-        <f aca="false">IF(C14&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>SELIC desde o pagamento</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="30" t="n">
-        <v>46037</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>125</v>
-      </c>
-      <c r="E15" s="30" t="n">
-        <f aca="false">MAX(C15,Resumo!$C$10)</f>
-        <v>46037</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E15+ABS(SELIC!$G$5:$G$18-E15))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E15+ABS(SELIC!$G$5:$G$18-E15))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.11035030540494</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <f aca="false">ROUND(D15*F15,2)</f>
-        <v>138.79</v>
-      </c>
-      <c r="H15" s="9" t="str">
-        <f aca="false">IF(C15&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>SELIC desde o pagamento</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
-        <v>46023</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="30" t="n">
-        <v>46037</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>125</v>
-      </c>
-      <c r="E16" s="30" t="n">
-        <f aca="false">MAX(C16,Resumo!$C$10)</f>
-        <v>46037</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <f aca="false">EXP(SUMPRODUCT(LN(1+SELIC!$B$5:$B$18*(((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E16+ABS(SELIC!$G$5:$G$18-E16))/2))+ABS((((SELIC!$H$5:$H$18+Resumo!$C$12-ABS(SELIC!$H$5:$H$18-Resumo!$C$12))/2)-((SELIC!$G$5:$G$18+E16+ABS(SELIC!$G$5:$G$18-E16))/2))))/2)/SELIC!$I$5:$I$18)))</f>
-        <v>1.11035030540494</v>
-      </c>
-      <c r="G16" s="7" t="n">
-        <f aca="false">ROUND(D16*F16,2)</f>
-        <v>138.79</v>
-      </c>
-      <c r="H16" s="9" t="str">
-        <f aca="false">IF(C16&lt;Resumo!$C$10,"Pago antes da citação – SELIC desde a citação","SELIC desde o pagamento")</f>
-        <v>SELIC desde o pagamento</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="16" t="n">
-        <f aca="false">SUM(D5:D16)</f>
-        <v>1500</v>
-      </c>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="16" t="n">
-        <f aca="false">SUM(G5:G16)</f>
-        <v>1689.18</v>
-      </c>
-      <c r="H17" s="14"/>
+      <c r="B14" s="14"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="16" t="n">
+        <f aca="false">SUM(D5:D13)</f>
+        <v>1125</v>
+      </c>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="16" t="n">
+        <f aca="false">SUM(G5:G13)</f>
+        <v>1263.45</v>
+      </c>
+      <c r="H14" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2332,4 +2315,241 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+    </row>
+    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1020</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>1020</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>122.65</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>122.65</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>122.65</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>9672.6</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>9672.6</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>9672.6</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>15.88</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>15.88</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <f aca="false">SUM(B5:B8)</f>
+        <v>10831.13</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <f aca="false">SUM(C5:C8)</f>
+        <v>10831.13</v>
+      </c>
+      <c r="D9" s="12" t="n">
+        <f aca="false">SUM(D5:D8)</f>
+        <v>10831.13</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="7" t="n">
+        <f aca="false">SUM(B9:D9)</f>
+        <v>32493.39</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="7" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="7" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="12" t="n">
+        <f aca="false">SUM(D12:D14)</f>
+        <v>33243.39</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="7" t="n">
+        <v>33247.41</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="12" t="n">
+        <f aca="false">D16-D15</f>
+        <v>4.02000000000407</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="31"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="31"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A19:D22"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Remove valores da multa e honorários do art. 523, § 1º (apuração posterior)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xsu4pqVYrCnjVCP87tgm6x
</commit_message>
<xml_diff>
--- a/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
+++ b/0800633-40.2025 - Maria dos Milagres/Planilha de cálculo - cumprimento de sentença.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="91">
   <si>
     <t xml:space="preserve">PLANILHA DE CÁLCULO – CUMPRIMENTO DE SENTENÇA</t>
   </si>
@@ -131,33 +131,6 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL DEVIDO PARA PAGAMENTO VOLUNTÁRIO (art. 523, caput, CPC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACRÉSCIMOS EM CASO DE NÃO PAGAMENTO EM 15 DIAS (art. 523, § 1º, CPC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Percentual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Art. 523, § 1º, CPC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Honorários advocatícios da fase de cumprimento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL APÓS O PRAZO SEM PAGAMENTO (TOTAL + MULTA + HONORÁRIOS)</t>
   </si>
   <si>
     <t xml:space="preserve">OBSERVAÇÕES</t>
@@ -301,6 +274,9 @@
   </si>
   <si>
     <t xml:space="preserve">Reconciliação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
   </si>
   <si>
     <t xml:space="preserve">Total do relatório até 01/09/2025</t>
@@ -520,7 +496,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -587,10 +563,6 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -943,7 +915,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1204,86 +1176,69 @@
       </c>
       <c r="F24" s="14"/>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2" t="s">
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+    </row>
+    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+    </row>
+    <row r="30" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="13" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E27" s="7" t="n">
-        <f aca="false">ROUND($E$24*D27,2)</f>
-        <v>4518.29</v>
-      </c>
-      <c r="F27" s="9" t="s">
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="13" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E28" s="7" t="n">
-        <f aca="false">ROUND($E$24*D28,2)</f>
-        <v>4518.29</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14"/>
-      <c r="B29" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="16" t="n">
-        <f aca="false">E24+E27+E28</f>
-        <v>54219.48</v>
-      </c>
-      <c r="F29" s="14"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B32" s="9"/>
       <c r="C32" s="9"/>
@@ -1293,7 +1248,7 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B33" s="9"/>
       <c r="C33" s="9"/>
@@ -1301,58 +1256,8 @@
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
     </row>
-    <row r="34" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-    </row>
-    <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-    </row>
-    <row r="36" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-    </row>
-    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B37" s="9"/>
-      <c r="C37" s="9"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-    </row>
-    <row r="38" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="18">
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="C9:F9"/>
@@ -1363,18 +1268,14 @@
     <mergeCell ref="C14:F14"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="C16:F16"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A35:F35"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A38:F38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
@@ -1405,528 +1306,528 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="A1" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
+      <c r="A2" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="20" t="n">
         <v>45901</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="21" t="n">
         <v>0.0122</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A5,0),Resumo!$C$12)-MAX(A5-1,Resumo!$C$10))/DAY(EOMONTH(A5,0))</f>
         <v>0</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A5,0),Resumo!$C$12)-MAX(A5-1,Resumo!$C$11))/DAY(EOMONTH(A5,0))</f>
         <v>0</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F5" s="9"/>
-      <c r="G5" s="24" t="n">
+      <c r="G5" s="23" t="n">
         <f aca="false">A5-1</f>
         <v>45900</v>
       </c>
-      <c r="H5" s="24" t="n">
+      <c r="H5" s="23" t="n">
         <f aca="false">EOMONTH(A5,0)</f>
         <v>45930</v>
       </c>
-      <c r="I5" s="25" t="n">
+      <c r="I5" s="24" t="n">
         <f aca="false">DAY(H5)</f>
         <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="n">
+      <c r="A6" s="20" t="n">
         <v>45931</v>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="21" t="n">
         <v>0.0128</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A6,0),Resumo!$C$12)-MAX(A6-1,Resumo!$C$10))/DAY(EOMONTH(A6,0))</f>
         <v>0</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A6,0),Resumo!$C$12)-MAX(A6-1,Resumo!$C$11))/DAY(EOMONTH(A6,0))</f>
         <v>0</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F6" s="9"/>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="23" t="n">
         <f aca="false">A6-1</f>
         <v>45930</v>
       </c>
-      <c r="H6" s="24" t="n">
+      <c r="H6" s="23" t="n">
         <f aca="false">EOMONTH(A6,0)</f>
         <v>45961</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="I6" s="24" t="n">
         <f aca="false">DAY(H6)</f>
         <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="20" t="n">
         <v>45962</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="21" t="n">
         <v>0.0105</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A7,0),Resumo!$C$12)-MAX(A7-1,Resumo!$C$10))/DAY(EOMONTH(A7,0))</f>
         <v>0.433333333333333</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A7,0),Resumo!$C$12)-MAX(A7-1,Resumo!$C$11))/DAY(EOMONTH(A7,0))</f>
         <v>0</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F7" s="9"/>
-      <c r="G7" s="24" t="n">
+      <c r="G7" s="23" t="n">
         <f aca="false">A7-1</f>
         <v>45961</v>
       </c>
-      <c r="H7" s="24" t="n">
+      <c r="H7" s="23" t="n">
         <f aca="false">EOMONTH(A7,0)</f>
         <v>45991</v>
       </c>
-      <c r="I7" s="25" t="n">
+      <c r="I7" s="24" t="n">
         <f aca="false">DAY(H7)</f>
         <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="n">
+      <c r="A8" s="20" t="n">
         <v>45992</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="21" t="n">
         <v>0.0122</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A8,0),Resumo!$C$12)-MAX(A8-1,Resumo!$C$10))/DAY(EOMONTH(A8,0))</f>
         <v>1</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A8,0),Resumo!$C$12)-MAX(A8-1,Resumo!$C$11))/DAY(EOMONTH(A8,0))</f>
         <v>0</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F8" s="9"/>
-      <c r="G8" s="24" t="n">
+      <c r="G8" s="23" t="n">
         <f aca="false">A8-1</f>
         <v>45991</v>
       </c>
-      <c r="H8" s="24" t="n">
+      <c r="H8" s="23" t="n">
         <f aca="false">EOMONTH(A8,0)</f>
         <v>46022</v>
       </c>
-      <c r="I8" s="25" t="n">
+      <c r="I8" s="24" t="n">
         <f aca="false">DAY(H8)</f>
         <v>31</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="20" t="n">
         <v>46023</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="21" t="n">
         <v>0.0116</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A9,0),Resumo!$C$12)-MAX(A9-1,Resumo!$C$10))/DAY(EOMONTH(A9,0))</f>
         <v>1</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A9,0),Resumo!$C$12)-MAX(A9-1,Resumo!$C$11))/DAY(EOMONTH(A9,0))</f>
         <v>0</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F9" s="9"/>
-      <c r="G9" s="24" t="n">
+      <c r="G9" s="23" t="n">
         <f aca="false">A9-1</f>
         <v>46022</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="23" t="n">
         <f aca="false">EOMONTH(A9,0)</f>
         <v>46053</v>
       </c>
-      <c r="I9" s="25" t="n">
+      <c r="I9" s="24" t="n">
         <f aca="false">DAY(H9)</f>
         <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="20" t="n">
         <v>46054</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="21" t="n">
         <v>0.01</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A10,0),Resumo!$C$12)-MAX(A10-1,Resumo!$C$10))/DAY(EOMONTH(A10,0))</f>
         <v>1</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A10,0),Resumo!$C$12)-MAX(A10-1,Resumo!$C$11))/DAY(EOMONTH(A10,0))</f>
         <v>0</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F10" s="9"/>
-      <c r="G10" s="24" t="n">
+      <c r="G10" s="23" t="n">
         <f aca="false">A10-1</f>
         <v>46053</v>
       </c>
-      <c r="H10" s="24" t="n">
+      <c r="H10" s="23" t="n">
         <f aca="false">EOMONTH(A10,0)</f>
         <v>46081</v>
       </c>
-      <c r="I10" s="25" t="n">
+      <c r="I10" s="24" t="n">
         <f aca="false">DAY(H10)</f>
         <v>28</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="20" t="n">
         <v>46082</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="21" t="n">
         <v>0.0121</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A11,0),Resumo!$C$12)-MAX(A11-1,Resumo!$C$10))/DAY(EOMONTH(A11,0))</f>
         <v>1</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A11,0),Resumo!$C$12)-MAX(A11-1,Resumo!$C$11))/DAY(EOMONTH(A11,0))</f>
         <v>0</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F11" s="9"/>
-      <c r="G11" s="24" t="n">
+      <c r="G11" s="23" t="n">
         <f aca="false">A11-1</f>
         <v>46081</v>
       </c>
-      <c r="H11" s="24" t="n">
+      <c r="H11" s="23" t="n">
         <f aca="false">EOMONTH(A11,0)</f>
         <v>46112</v>
       </c>
-      <c r="I11" s="25" t="n">
+      <c r="I11" s="24" t="n">
         <f aca="false">DAY(H11)</f>
         <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="20" t="n">
         <v>46113</v>
       </c>
-      <c r="B12" s="22" t="n">
+      <c r="B12" s="21" t="n">
         <v>0.0109</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A12,0),Resumo!$C$12)-MAX(A12-1,Resumo!$C$10))/DAY(EOMONTH(A12,0))</f>
         <v>1</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A12,0),Resumo!$C$12)-MAX(A12-1,Resumo!$C$11))/DAY(EOMONTH(A12,0))</f>
         <v>0</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F12" s="9"/>
-      <c r="G12" s="24" t="n">
+      <c r="G12" s="23" t="n">
         <f aca="false">A12-1</f>
         <v>46112</v>
       </c>
-      <c r="H12" s="24" t="n">
+      <c r="H12" s="23" t="n">
         <f aca="false">EOMONTH(A12,0)</f>
         <v>46142</v>
       </c>
-      <c r="I12" s="25" t="n">
+      <c r="I12" s="24" t="n">
         <f aca="false">DAY(H12)</f>
         <v>30</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="20" t="n">
         <v>46143</v>
       </c>
-      <c r="B13" s="22" t="n">
+      <c r="B13" s="21" t="n">
         <v>0.0107</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A13,0),Resumo!$C$12)-MAX(A13-1,Resumo!$C$10))/DAY(EOMONTH(A13,0))</f>
         <v>1</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A13,0),Resumo!$C$12)-MAX(A13-1,Resumo!$C$11))/DAY(EOMONTH(A13,0))</f>
         <v>0</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F13" s="9"/>
-      <c r="G13" s="24" t="n">
+      <c r="G13" s="23" t="n">
         <f aca="false">A13-1</f>
         <v>46142</v>
       </c>
-      <c r="H13" s="24" t="n">
+      <c r="H13" s="23" t="n">
         <f aca="false">EOMONTH(A13,0)</f>
         <v>46173</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="I13" s="24" t="n">
         <f aca="false">DAY(H13)</f>
         <v>31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="20" t="n">
         <v>46174</v>
       </c>
-      <c r="B14" s="22" t="n">
+      <c r="B14" s="21" t="n">
         <v>0.0112</v>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A14,0),Resumo!$C$12)-MAX(A14-1,Resumo!$C$10))/DAY(EOMONTH(A14,0))</f>
         <v>1</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A14,0),Resumo!$C$12)-MAX(A14-1,Resumo!$C$11))/DAY(EOMONTH(A14,0))</f>
         <v>0</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F14" s="9"/>
-      <c r="G14" s="24" t="n">
+      <c r="G14" s="23" t="n">
         <f aca="false">A14-1</f>
         <v>46173</v>
       </c>
-      <c r="H14" s="24" t="n">
+      <c r="H14" s="23" t="n">
         <f aca="false">EOMONTH(A14,0)</f>
         <v>46203</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="I14" s="24" t="n">
         <f aca="false">DAY(H14)</f>
         <v>30</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="20" t="n">
         <v>46204</v>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="21" t="n">
         <v>0.0122</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A15,0),Resumo!$C$12)-MAX(A15-1,Resumo!$C$10))/DAY(EOMONTH(A15,0))</f>
         <v>1</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A15,0),Resumo!$C$12)-MAX(A15-1,Resumo!$C$11))/DAY(EOMONTH(A15,0))</f>
         <v>0.032258064516129</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F15" s="9"/>
-      <c r="G15" s="24" t="n">
+      <c r="G15" s="23" t="n">
         <f aca="false">A15-1</f>
         <v>46203</v>
       </c>
-      <c r="H15" s="24" t="n">
+      <c r="H15" s="23" t="n">
         <f aca="false">EOMONTH(A15,0)</f>
         <v>46234</v>
       </c>
-      <c r="I15" s="25" t="n">
+      <c r="I15" s="24" t="n">
         <f aca="false">DAY(H15)</f>
         <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="20" t="n">
         <v>46235</v>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="21" t="n">
         <v>0.0109</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A16,0),Resumo!$C$12)-MAX(A16-1,Resumo!$C$10))/DAY(EOMONTH(A16,0))</f>
         <v>1</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A16,0),Resumo!$C$12)-MAX(A16-1,Resumo!$C$11))/DAY(EOMONTH(A16,0))</f>
         <v>1</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F16" s="9"/>
-      <c r="G16" s="24" t="n">
+      <c r="G16" s="23" t="n">
         <f aca="false">A16-1</f>
         <v>46234</v>
       </c>
-      <c r="H16" s="24" t="n">
+      <c r="H16" s="23" t="n">
         <f aca="false">EOMONTH(A16,0)</f>
         <v>46265</v>
       </c>
-      <c r="I16" s="25" t="n">
+      <c r="I16" s="24" t="n">
         <f aca="false">DAY(H16)</f>
         <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="20" t="n">
         <v>46266</v>
       </c>
-      <c r="B17" s="22" t="n">
+      <c r="B17" s="21" t="n">
         <v>0.0108</v>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A17,0),Resumo!$C$12)-MAX(A17-1,Resumo!$C$10))/DAY(EOMONTH(A17,0))</f>
         <v>1</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A17,0),Resumo!$C$12)-MAX(A17-1,Resumo!$C$11))/DAY(EOMONTH(A17,0))</f>
         <v>1</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F17" s="9"/>
-      <c r="G17" s="24" t="n">
+      <c r="G17" s="23" t="n">
         <f aca="false">A17-1</f>
         <v>46265</v>
       </c>
-      <c r="H17" s="24" t="n">
+      <c r="H17" s="23" t="n">
         <f aca="false">EOMONTH(A17,0)</f>
         <v>46295</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="I17" s="24" t="n">
         <f aca="false">DAY(H17)</f>
         <v>30</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="20" t="n">
         <v>46296</v>
       </c>
-      <c r="B18" s="26" t="n">
+      <c r="B18" s="25" t="n">
         <v>0.0108</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$10))/DAY(EOMONTH(A18,0))</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="22" t="n">
         <f aca="false">MAX(0,MIN(EOMONTH(A18,0),Resumo!$C$12)-MAX(A18-1,Resumo!$C$11))/DAY(EOMONTH(A18,0))</f>
         <v>0.967741935483871</v>
       </c>
-      <c r="E18" s="27" t="s">
-        <v>65</v>
+      <c r="E18" s="26" t="s">
+        <v>56</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G18" s="24" t="n">
+        <v>57</v>
+      </c>
+      <c r="G18" s="23" t="n">
         <f aca="false">A18-1</f>
         <v>46295</v>
       </c>
-      <c r="H18" s="24" t="n">
+      <c r="H18" s="23" t="n">
         <f aca="false">EOMONTH(A18,0)</f>
         <v>46326</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="I18" s="24" t="n">
         <f aca="false">DAY(H18)</f>
         <v>31</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B20" s="11"/>
-      <c r="C20" s="28" t="n">
+      <c r="C20" s="27" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*C5:C18)))</f>
         <v>1.13530961958417</v>
       </c>
-      <c r="D20" s="28" t="n">
+      <c r="D20" s="27" t="n">
         <f aca="false">EXP(SUMPRODUCT(LN(1+$B$5:$B$18*D5:D18)))</f>
         <v>1.03290370093909</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B21" s="11"/>
-      <c r="C21" s="29" t="n">
+      <c r="C21" s="28" t="n">
         <f aca="false">C20-1</f>
         <v>0.135309619584169</v>
       </c>
-      <c r="D21" s="29" t="n">
+      <c r="D21" s="28" t="n">
         <f aca="false">D20-1</f>
         <v>0.0329037009390918</v>
       </c>
@@ -1965,44 +1866,44 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="A1" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
+      <c r="A2" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>18</v>
@@ -2011,23 +1912,23 @@
         <v>19</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="20" t="n">
         <v>45962</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="30" t="n">
+        <v>67</v>
+      </c>
+      <c r="C5" s="29" t="n">
         <v>45976</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="29" t="n">
         <f aca="false">MAX(C5,Resumo!$C$10)</f>
         <v>45978</v>
       </c>
@@ -2045,19 +1946,19 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="n">
+      <c r="A6" s="20" t="n">
         <v>45962</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C6" s="30" t="n">
+        <v>68</v>
+      </c>
+      <c r="C6" s="29" t="n">
         <v>45976</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="29" t="n">
         <f aca="false">MAX(C6,Resumo!$C$10)</f>
         <v>45978</v>
       </c>
@@ -2075,19 +1976,19 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="20" t="n">
         <v>45962</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="30" t="n">
+        <v>69</v>
+      </c>
+      <c r="C7" s="29" t="n">
         <v>45976</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="29" t="n">
         <f aca="false">MAX(C7,Resumo!$C$10)</f>
         <v>45978</v>
       </c>
@@ -2105,19 +2006,19 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="n">
+      <c r="A8" s="20" t="n">
         <v>45992</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C8" s="30" t="n">
+        <v>67</v>
+      </c>
+      <c r="C8" s="29" t="n">
         <v>46006</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="29" t="n">
         <f aca="false">MAX(C8,Resumo!$C$10)</f>
         <v>46006</v>
       </c>
@@ -2135,19 +2036,19 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="20" t="n">
         <v>45992</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C9" s="30" t="n">
+        <v>68</v>
+      </c>
+      <c r="C9" s="29" t="n">
         <v>46006</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E9" s="29" t="n">
         <f aca="false">MAX(C9,Resumo!$C$10)</f>
         <v>46006</v>
       </c>
@@ -2165,19 +2066,19 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="20" t="n">
         <v>45992</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="30" t="n">
+        <v>69</v>
+      </c>
+      <c r="C10" s="29" t="n">
         <v>46006</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="29" t="n">
         <f aca="false">MAX(C10,Resumo!$C$10)</f>
         <v>46006</v>
       </c>
@@ -2195,19 +2096,19 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="20" t="n">
         <v>46023</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="30" t="n">
+        <v>67</v>
+      </c>
+      <c r="C11" s="29" t="n">
         <v>46037</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E11" s="30" t="n">
+      <c r="E11" s="29" t="n">
         <f aca="false">MAX(C11,Resumo!$C$10)</f>
         <v>46037</v>
       </c>
@@ -2225,19 +2126,19 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="20" t="n">
         <v>46023</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C12" s="30" t="n">
+        <v>68</v>
+      </c>
+      <c r="C12" s="29" t="n">
         <v>46037</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E12" s="30" t="n">
+      <c r="E12" s="29" t="n">
         <f aca="false">MAX(C12,Resumo!$C$10)</f>
         <v>46037</v>
       </c>
@@ -2255,19 +2156,19 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="20" t="n">
         <v>46023</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="30" t="n">
+        <v>69</v>
+      </c>
+      <c r="C13" s="29" t="n">
         <v>46037</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>125</v>
       </c>
-      <c r="E13" s="30" t="n">
+      <c r="E13" s="29" t="n">
         <f aca="false">MAX(C13,Resumo!$C$10)</f>
         <v>46037</v>
       </c>
@@ -2286,7 +2187,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -2330,38 +2231,38 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
+      <c r="A1" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
+      <c r="A2" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B5" s="7" t="n">
         <v>1020</v>
@@ -2375,7 +2276,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>122.65</v>
@@ -2389,7 +2290,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>9672.6</v>
@@ -2403,7 +2304,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>15.88</v>
@@ -2417,7 +2318,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">SUM(B5:B8)</f>
@@ -2434,17 +2335,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
-        <v>38</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
@@ -2455,7 +2356,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -2465,7 +2366,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
@@ -2475,7 +2376,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -2486,7 +2387,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -2496,7 +2397,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2506,30 +2407,30 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
+      <c r="A19" s="30" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="31"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="31"/>
+      <c r="A20" s="30"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="31"/>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="31"/>
+      <c r="A21" s="30"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="31"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="31"/>
-      <c r="D22" s="31"/>
+      <c r="A22" s="30"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>